<commit_message>
feat: add comprehensive 2026 OBE curriculum revision files and update AGENTS.md
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/004_MATRIKS_KETERLACAKAN_OBE_VMTS_PEO_PL_CPL_MK.xlsx
+++ b/KURIKULUM2026_REVISI/004_MATRIKS_KETERLACAKAN_OBE_VMTS_PEO_PL_CPL_MK.xlsx
@@ -3521,7 +3521,7 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>`STI-626`</t>
+          <t>`STI-726`</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>`STI-627`</t>
+          <t>`STI-727`</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
@@ -4204,7 +4204,7 @@
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>`STI-624`</t>
+          <t>`STI-726`</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
@@ -4263,7 +4263,7 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>`STI-625`</t>
+          <t>`STI-727`</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
@@ -6293,7 +6293,7 @@
       </c>
       <c r="D131" s="8" t="inlineStr">
         <is>
-          <t>`STI-306`, `STI-627`</t>
+          <t>`STI-306`, `STI-727`</t>
         </is>
       </c>
       <c r="E131" s="8" t="inlineStr">
@@ -6453,7 +6453,7 @@
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>`STI-306`, `STI-625`</t>
+          <t>`STI-306`, `STI-727`</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t>`STI-311`, `STI-416`, `STI-522`, `STI-627`</t>
+          <t>`STI-311`, `STI-416`, `STI-522`, `STI-727`</t>
         </is>
       </c>
       <c r="D139" s="8" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t>`STI-307`, `STI-414`, `STI-624`, `STA-602`, `STA-702`</t>
+          <t>`STI-307`, `STI-414`, `STI-726`, `STA-602`, `STA-702`</t>
         </is>
       </c>
       <c r="D143" s="8" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t>`STI-413`, `STI-626`, `STA-701`</t>
+          <t>`STI-413`, `STI-726`, `STA-701`</t>
         </is>
       </c>
       <c r="D145" s="8" t="inlineStr">
@@ -6773,7 +6773,7 @@
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>`STI-627`, `STC-702`</t>
+          <t>`STI-727`, `STC-702`</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="D147" s="8" t="inlineStr">
         <is>
-          <t>`STI-418`, `STI-625`, `STB-701`</t>
+          <t>`STI-418`, `STI-727`, `STB-701`</t>
         </is>
       </c>
       <c r="E147" s="8" t="inlineStr">
@@ -6941,7 +6941,7 @@
       </c>
       <c r="C153" s="8" t="inlineStr">
         <is>
-          <t>`STI-307`, `STI-413`, `STI-414`, `STI-626`, `STI-624`</t>
+          <t>`STI-307`, `STI-413`, `STI-414`, `STI-726`, `STI-726`</t>
         </is>
       </c>
       <c r="D153" s="8" t="inlineStr">
@@ -7005,7 +7005,7 @@
       </c>
       <c r="C155" s="8" t="inlineStr">
         <is>
-          <t>`STI-311`, `STI-416`, `STI-522`, `STI-627`</t>
+          <t>`STI-311`, `STI-416`, `STI-522`, `STI-727`</t>
         </is>
       </c>
       <c r="D155" s="8" t="inlineStr">
@@ -7101,7 +7101,7 @@
       </c>
       <c r="C158" s="7" t="inlineStr">
         <is>
-          <t>`STI-624`, `STI-627`, `FST-610`</t>
+          <t>`STI-726`, `STI-727`, `FST-610`</t>
         </is>
       </c>
       <c r="D158" s="7" t="inlineStr">
@@ -7229,7 +7229,7 @@
       </c>
       <c r="C162" s="7" t="inlineStr">
         <is>
-          <t>`STI-309`, `STI-416`, `STI-627`</t>
+          <t>`STI-309`, `STI-416`, `STI-727`</t>
         </is>
       </c>
       <c r="D162" s="7" t="inlineStr">
@@ -9280,7 +9280,7 @@
       </c>
       <c r="B209" s="8" t="inlineStr">
         <is>
-          <t>`STI-624`</t>
+          <t>`STI-726`</t>
         </is>
       </c>
       <c r="C209" s="8" t="inlineStr">
@@ -9327,7 +9327,7 @@
       </c>
       <c r="B210" s="7" t="inlineStr">
         <is>
-          <t>`STI-625`</t>
+          <t>`STI-727`</t>
         </is>
       </c>
       <c r="C210" s="7" t="inlineStr">
@@ -9374,7 +9374,7 @@
       </c>
       <c r="B211" s="8" t="inlineStr">
         <is>
-          <t>`STI-626`</t>
+          <t>`STI-726`</t>
         </is>
       </c>
       <c r="C211" s="8" t="inlineStr">
@@ -9421,7 +9421,7 @@
       </c>
       <c r="B212" s="7" t="inlineStr">
         <is>
-          <t>`STI-627`</t>
+          <t>`STI-727`</t>
         </is>
       </c>
       <c r="C212" s="7" t="inlineStr">

</xml_diff>